<commit_message>
Fase 155, PR 3: plantilla de Flujo de Llamadas = reporte de Wolkvox
- PLANTILLA_FLUJO_LLAMADAS.xlsx con las 15 columnas del reporte de la cola
  de Wolkvox en su orden (se agrega ABANDON, reconocida pero nunca leida).
- INSTRUCCIONES y ficha: "Nivel de atencion y tasa de abandono los calcula
  el sistema; no hace falta llenarlos." Ficha regenerada con el generador.
- v1.54.5 y CHANGELOG.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/plantillas/PLANTILLA_FLUJO_LLAMADAS.xlsx
+++ b/server/plantillas/PLANTILLA_FLUJO_LLAMADAS.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:O1"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -412,8 +412,9 @@
     <col min="10" max="10" width="14.83203125" customWidth="1"/>
     <col min="11" max="11" width="14.83203125" customWidth="1"/>
     <col min="12" max="12" width="14.83203125" customWidth="1"/>
-    <col min="13" max="13" width="19.83203125" customWidth="1"/>
-    <col min="14" max="14" width="17.83203125" customWidth="1"/>
+    <col min="13" max="13" width="14.83203125" customWidth="1"/>
+    <col min="14" max="14" width="19.83203125" customWidth="1"/>
+    <col min="15" max="15" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -442,34 +443,37 @@
         <v>SERVICE_LEVEL_30SEC</v>
       </c>
       <c r="I1" t="str">
+        <v>ABANDON</v>
+      </c>
+      <c r="J1" t="str">
         <v>ASA</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>ATA</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>WAIT_TIME</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>AHT</v>
       </c>
-      <c r="M1" t="str">
+      <c r="N1" t="str">
         <v>NIVEL DE ATENCION</v>
       </c>
-      <c r="N1" t="str">
+      <c r="O1" t="str">
         <v>TASA DE ABNDONO</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:N1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E23"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -501,117 +505,108 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Cómo se sube</v>
+        <v>Cálculos</v>
       </c>
       <c r="B4" t="str">
-        <v>Cargar Datos → cliente → este módulo. El sistema reconoce el archivo por sus columnas, no por el nombre de la hoja ni del archivo.</v>
+        <v>Nivel de atención y tasa de abandono los calcula el sistema; no hace falta llenarlos.</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
+        <v>Cómo se sube</v>
+      </c>
+      <c r="B5" t="str">
+        <v>Cargar Datos → cliente → este módulo. El sistema reconoce el archivo por sus columnas, no por el nombre de la hoja ni del archivo.</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
         <v>Importante</v>
       </c>
-      <c r="B5" t="str">
+      <c r="B6" t="str">
         <v>No cambie los nombres de las columnas. Los ejemplos de abajo son inventados: no los copie a la hoja de datos.</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Columna</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Obligatoria</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Qué va</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Ejemplo (inventado)</v>
-      </c>
-      <c r="E7" t="str">
-        <v>También se acepta como</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>SKILL_NAME</v>
+        <v>Columna</v>
       </c>
       <c r="B8" t="str">
-        <v>Sí</v>
+        <v>Obligatoria</v>
       </c>
       <c r="C8" t="str">
-        <v>Línea o skill de Wolkvox (Mobilize: "TIPO DE LINEA").</v>
+        <v>Qué va</v>
       </c>
       <c r="D8" t="str">
-        <v>SKILL SAC</v>
+        <v>Ejemplo (inventado)</v>
       </c>
       <c r="E8" t="str">
-        <v>TIPO DE LINEA</v>
+        <v>También se acepta como</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>DATE</v>
+        <v>SKILL_NAME</v>
       </c>
       <c r="B9" t="str">
         <v>Sí</v>
       </c>
       <c r="C9" t="str">
-        <v>Día (Mobilize: "DÍA").</v>
+        <v>Línea o skill de Wolkvox (Mobilize: "TIPO DE LINEA").</v>
       </c>
       <c r="D9" t="str">
-        <v>2026-08-01</v>
+        <v>SKILL SAC</v>
       </c>
       <c r="E9" t="str">
-        <v>DÍA, DIA</v>
+        <v>TIPO DE LINEA</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>TOTAL LLAMADAS</v>
+        <v>DATE</v>
       </c>
       <c r="B10" t="str">
         <v>Sí</v>
       </c>
       <c r="C10" t="str">
-        <v>Llamadas que entraron a la cola ese día (Mobilize: "LLAMADAS INGRESADAS").</v>
-      </c>
-      <c r="D10">
-        <v>120</v>
+        <v>Día (Mobilize: "DÍA").</v>
+      </c>
+      <c r="D10" t="str">
+        <v>2026-08-01</v>
       </c>
       <c r="E10" t="str">
-        <v>LLAMADAS INGRESADAS</v>
+        <v>DÍA, DIA</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>LLAMADAS CONTESTADAS</v>
+        <v>TOTAL LLAMADAS</v>
       </c>
       <c r="B11" t="str">
         <v>Sí</v>
       </c>
       <c r="C11" t="str">
-        <v>Llamadas atendidas.</v>
+        <v>Llamadas que entraron a la cola ese día (Mobilize: "LLAMADAS INGRESADAS").</v>
       </c>
       <c r="D11">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="E11" t="str">
-        <v/>
+        <v>LLAMADAS INGRESADAS</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>LLAMADAS ABANDONADAS</v>
+        <v>LLAMADAS CONTESTADAS</v>
       </c>
       <c r="B12" t="str">
-        <v>No</v>
+        <v>Sí</v>
       </c>
       <c r="C12" t="str">
-        <v>Llamadas que colgaron antes de ser atendidas.</v>
+        <v>Llamadas atendidas.</v>
       </c>
       <c r="D12">
-        <v>8</v>
+        <v>112</v>
       </c>
       <c r="E12" t="str">
         <v/>
@@ -619,16 +614,16 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>SERVICE_LEVEL_10SEC</v>
+        <v>LLAMADAS ABANDONADAS</v>
       </c>
       <c r="B13" t="str">
         <v>No</v>
       </c>
       <c r="C13" t="str">
-        <v>% atendidas en 10 s.</v>
+        <v>Llamadas que colgaron antes de ser atendidas.</v>
       </c>
       <c r="D13">
-        <v>0.85</v>
+        <v>8</v>
       </c>
       <c r="E13" t="str">
         <v/>
@@ -636,50 +631,50 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>SERVICE_LEVEL_20SEC</v>
+        <v>SERVICE_LEVEL_10SEC</v>
       </c>
       <c r="B14" t="str">
         <v>No</v>
       </c>
       <c r="C14" t="str">
-        <v>% atendidas en 20 s (Mobilize: "NIVEL DE SERVICIO 80 - 20").</v>
+        <v>% atendidas en 10 s.</v>
       </c>
       <c r="D14">
-        <v>0.9</v>
+        <v>0.85</v>
       </c>
       <c r="E14" t="str">
-        <v>NIVEL DE SERVICIO 80 - 20</v>
+        <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>SERVICE_LEVEL_30SEC</v>
+        <v>SERVICE_LEVEL_20SEC</v>
       </c>
       <c r="B15" t="str">
         <v>No</v>
       </c>
       <c r="C15" t="str">
-        <v>% atendidas en 30 s.</v>
+        <v>% atendidas en 20 s (Mobilize: "NIVEL DE SERVICIO 80 - 20").</v>
       </c>
       <c r="D15">
-        <v>0.93</v>
+        <v>0.9</v>
       </c>
       <c r="E15" t="str">
-        <v/>
+        <v>NIVEL DE SERVICIO 80 - 20</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>ASA</v>
+        <v>SERVICE_LEVEL_30SEC</v>
       </c>
       <c r="B16" t="str">
         <v>No</v>
       </c>
       <c r="C16" t="str">
-        <v>Tiempo promedio de respuesta (segundos o mm:ss).</v>
+        <v>% atendidas en 30 s.</v>
       </c>
       <c r="D16">
-        <v>12</v>
+        <v>0.93</v>
       </c>
       <c r="E16" t="str">
         <v/>
@@ -687,16 +682,16 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>ATA</v>
+        <v>ABANDON</v>
       </c>
       <c r="B17" t="str">
         <v>No</v>
       </c>
       <c r="C17" t="str">
-        <v>Tiempo promedio hasta el abandono.</v>
+        <v>% de abandono que reporta Wolkvox. Se deja como viene: el sistema no la usa (calcula la tasa de abandono con las llamadas).</v>
       </c>
       <c r="D17">
-        <v>30</v>
+        <v>0.07</v>
       </c>
       <c r="E17" t="str">
         <v/>
@@ -704,16 +699,16 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>WAIT_TIME</v>
+        <v>ASA</v>
       </c>
       <c r="B18" t="str">
         <v>No</v>
       </c>
       <c r="C18" t="str">
-        <v>Tiempo de espera.</v>
+        <v>Tiempo promedio de respuesta (segundos o mm:ss).</v>
       </c>
       <c r="D18">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E18" t="str">
         <v/>
@@ -721,16 +716,16 @@
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>AHT</v>
+        <v>ATA</v>
       </c>
       <c r="B19" t="str">
         <v>No</v>
       </c>
       <c r="C19" t="str">
-        <v>Tiempo promedio de atención.</v>
+        <v>Tiempo promedio hasta el abandono.</v>
       </c>
       <c r="D19">
-        <v>210</v>
+        <v>30</v>
       </c>
       <c r="E19" t="str">
         <v/>
@@ -738,16 +733,16 @@
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>NIVEL DE ATENCION</v>
+        <v>WAIT_TIME</v>
       </c>
       <c r="B20" t="str">
         <v>No</v>
       </c>
       <c r="C20" t="str">
-        <v>% de llamadas atendidas.</v>
+        <v>Tiempo de espera.</v>
       </c>
       <c r="D20">
-        <v>0.93</v>
+        <v>15</v>
       </c>
       <c r="E20" t="str">
         <v/>
@@ -755,24 +750,58 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
+        <v>AHT</v>
+      </c>
+      <c r="B21" t="str">
+        <v>No</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Tiempo promedio de atención.</v>
+      </c>
+      <c r="D21">
+        <v>210</v>
+      </c>
+      <c r="E21" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>NIVEL DE ATENCION</v>
+      </c>
+      <c r="B22" t="str">
+        <v>No</v>
+      </c>
+      <c r="C22" t="str">
+        <v>No hace falta llenarla: el sistema la calcula (contestadas ÷ ingresadas). Si viene llena, no se usa.</v>
+      </c>
+      <c r="D22" t="str">
+        <v/>
+      </c>
+      <c r="E22" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
         <v>TASA DE ABNDONO</v>
       </c>
-      <c r="B21" t="str">
-        <v>No</v>
-      </c>
-      <c r="C21" t="str">
-        <v>% de abandono (así viene escrito de Wolkvox; Mobilize: "% ABANDONO").</v>
-      </c>
-      <c r="D21">
-        <v>0.07</v>
-      </c>
-      <c r="E21" t="str">
+      <c r="B23" t="str">
+        <v>No</v>
+      </c>
+      <c r="C23" t="str">
+        <v>No hace falta llenarla: el sistema la calcula (abandonadas ÷ ingresadas). Si viene llena, no se usa. (Así viene escrito de Wolkvox; Mobilize: "% ABANDONO").</v>
+      </c>
+      <c r="D23" t="str">
+        <v/>
+      </c>
+      <c r="E23" t="str">
         <v>% ABANDONO</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E23"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fase 159 (plantilla): Flujo de Llamadas con los encabezados nativos de Wolkvox (v1.57.7)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/plantillas/PLANTILLA_FLUJO_LLAMADAS.xlsx
+++ b/server/plantillas/PLANTILLA_FLUJO_LLAMADAS.xlsx
@@ -398,13 +398,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:M1"/>
   <cols>
     <col min="1" max="1" width="14.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
-    <col min="3" max="3" width="16.83203125" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="15.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="15.83203125" customWidth="1"/>
     <col min="6" max="6" width="21.83203125" customWidth="1"/>
     <col min="7" max="7" width="21.83203125" customWidth="1"/>
     <col min="8" max="8" width="21.83203125" customWidth="1"/>
@@ -413,8 +413,6 @@
     <col min="11" max="11" width="14.83203125" customWidth="1"/>
     <col min="12" max="12" width="14.83203125" customWidth="1"/>
     <col min="13" max="13" width="14.83203125" customWidth="1"/>
-    <col min="14" max="14" width="19.83203125" customWidth="1"/>
-    <col min="15" max="15" width="17.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -425,13 +423,13 @@
         <v>DATE</v>
       </c>
       <c r="C1" t="str">
-        <v>TOTAL LLAMADAS</v>
+        <v>INBOUND_CALLS</v>
       </c>
       <c r="D1" t="str">
-        <v>LLAMADAS CONTESTADAS</v>
+        <v>ANSWER_CALLS</v>
       </c>
       <c r="E1" t="str">
-        <v>LLAMADAS ABANDONADAS</v>
+        <v>ABANDON_CALLS</v>
       </c>
       <c r="F1" t="str">
         <v>SERVICE_LEVEL_10SEC</v>
@@ -457,23 +455,17 @@
       <c r="M1" t="str">
         <v>AHT</v>
       </c>
-      <c r="N1" t="str">
-        <v>NIVEL DE ATENCION</v>
-      </c>
-      <c r="O1" t="str">
-        <v>TASA DE ABNDONO</v>
-      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E21"/>
   <cols>
     <col min="1" max="1" width="26.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -552,7 +544,7 @@
         <v>Sí</v>
       </c>
       <c r="C9" t="str">
-        <v>Línea o skill de Wolkvox (Mobilize: "TIPO DE LINEA").</v>
+        <v>Línea o skill de Wolkvox.</v>
       </c>
       <c r="D9" t="str">
         <v>SKILL SAC</v>
@@ -569,7 +561,7 @@
         <v>Sí</v>
       </c>
       <c r="C10" t="str">
-        <v>Día (Mobilize: "DÍA").</v>
+        <v>Día.</v>
       </c>
       <c r="D10" t="str">
         <v>2026-08-01</v>
@@ -580,24 +572,24 @@
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>TOTAL LLAMADAS</v>
+        <v>INBOUND_CALLS</v>
       </c>
       <c r="B11" t="str">
         <v>Sí</v>
       </c>
       <c r="C11" t="str">
-        <v>Llamadas que entraron a la cola ese día (Mobilize: "LLAMADAS INGRESADAS").</v>
+        <v>Llamadas que entraron a la cola ese día (ingresadas).</v>
       </c>
       <c r="D11">
         <v>120</v>
       </c>
       <c r="E11" t="str">
-        <v>LLAMADAS INGRESADAS</v>
+        <v>TOTAL LLAMADAS, LLAMADAS INGRESADAS</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>LLAMADAS CONTESTADAS</v>
+        <v>ANSWER_CALLS</v>
       </c>
       <c r="B12" t="str">
         <v>Sí</v>
@@ -609,12 +601,12 @@
         <v>112</v>
       </c>
       <c r="E12" t="str">
-        <v/>
+        <v>LLAMADAS CONTESTADAS</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>LLAMADAS ABANDONADAS</v>
+        <v>ABANDON_CALLS</v>
       </c>
       <c r="B13" t="str">
         <v>No</v>
@@ -626,7 +618,7 @@
         <v>8</v>
       </c>
       <c r="E13" t="str">
-        <v/>
+        <v>LLAMADAS ABANDONADAS</v>
       </c>
     </row>
     <row r="14">
@@ -637,10 +629,10 @@
         <v>No</v>
       </c>
       <c r="C14" t="str">
-        <v>% atendidas en 10 s.</v>
-      </c>
-      <c r="D14">
-        <v>0.85</v>
+        <v>% atendidas en 10 s. Puede venir como texto ("66.67 %").</v>
+      </c>
+      <c r="D14" t="str">
+        <v>66.67 %</v>
       </c>
       <c r="E14" t="str">
         <v/>
@@ -654,10 +646,10 @@
         <v>No</v>
       </c>
       <c r="C15" t="str">
-        <v>% atendidas en 20 s (Mobilize: "NIVEL DE SERVICIO 80 - 20").</v>
-      </c>
-      <c r="D15">
-        <v>0.9</v>
+        <v>% atendidas en 20 s (nivel de servicio 80 - 20).</v>
+      </c>
+      <c r="D15" t="str">
+        <v>80.00 %</v>
       </c>
       <c r="E15" t="str">
         <v>NIVEL DE SERVICIO 80 - 20</v>
@@ -673,8 +665,8 @@
       <c r="C16" t="str">
         <v>% atendidas en 30 s.</v>
       </c>
-      <c r="D16">
-        <v>0.93</v>
+      <c r="D16" t="str">
+        <v>93.00 %</v>
       </c>
       <c r="E16" t="str">
         <v/>
@@ -690,8 +682,8 @@
       <c r="C17" t="str">
         <v>% de abandono que reporta Wolkvox. Se deja como viene: el sistema no la usa (calcula la tasa de abandono con las llamadas).</v>
       </c>
-      <c r="D17">
-        <v>0.07</v>
+      <c r="D17" t="str">
+        <v>0.00%</v>
       </c>
       <c r="E17" t="str">
         <v/>
@@ -705,10 +697,10 @@
         <v>No</v>
       </c>
       <c r="C18" t="str">
-        <v>Tiempo promedio de respuesta (segundos o mm:ss).</v>
-      </c>
-      <c r="D18">
-        <v>12</v>
+        <v>Tiempo promedio de respuesta (segundos, también como texto "11.00").</v>
+      </c>
+      <c r="D18" t="str">
+        <v>11.00</v>
       </c>
       <c r="E18" t="str">
         <v/>
@@ -724,8 +716,8 @@
       <c r="C19" t="str">
         <v>Tiempo promedio hasta el abandono.</v>
       </c>
-      <c r="D19">
-        <v>30</v>
+      <c r="D19" t="str">
+        <v>30.00</v>
       </c>
       <c r="E19" t="str">
         <v/>
@@ -739,10 +731,10 @@
         <v>No</v>
       </c>
       <c r="C20" t="str">
-        <v>Tiempo de espera.</v>
-      </c>
-      <c r="D20">
-        <v>15</v>
+        <v>Tiempo de espera (hora de Excel o segundos).</v>
+      </c>
+      <c r="D20" t="str">
+        <v>0:00:15</v>
       </c>
       <c r="E20" t="str">
         <v/>
@@ -756,52 +748,18 @@
         <v>No</v>
       </c>
       <c r="C21" t="str">
-        <v>Tiempo promedio de atención.</v>
-      </c>
-      <c r="D21">
-        <v>210</v>
+        <v>Tiempo promedio de atención (hora de Excel o segundos). "----" o vacío = sin dato, nunca 0.</v>
+      </c>
+      <c r="D21" t="str">
+        <v>0:03:30</v>
       </c>
       <c r="E21" t="str">
         <v/>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>NIVEL DE ATENCION</v>
-      </c>
-      <c r="B22" t="str">
-        <v>No</v>
-      </c>
-      <c r="C22" t="str">
-        <v>No hace falta llenarla: el sistema la calcula (contestadas ÷ ingresadas). Si viene llena, no se usa.</v>
-      </c>
-      <c r="D22" t="str">
-        <v/>
-      </c>
-      <c r="E22" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>TASA DE ABNDONO</v>
-      </c>
-      <c r="B23" t="str">
-        <v>No</v>
-      </c>
-      <c r="C23" t="str">
-        <v>No hace falta llenarla: el sistema la calcula (abandonadas ÷ ingresadas). Si viene llena, no se usa. (Así viene escrito de Wolkvox; Mobilize: "% ABANDONO").</v>
-      </c>
-      <c r="D23" t="str">
-        <v/>
-      </c>
-      <c r="E23" t="str">
-        <v>% ABANDONO</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E21"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>